<commit_message>
security: scrub member emails, add SRI, harden links and Actions
- updates/members: replace real member emails with TBD in committed
  spreadsheets; they were publicly downloadable via the Pages deploy
- all pages: add SRI integrity hash to the Bootstrap JS bundle (CSS
  already had one); hash verified against the live CDN file
- index/mariamguizani: add rel=noopener to target=_blank links
- publication.html: route paper links through safeUrl() allowing only
  http(s) URLs, escaped before href interpolation
- workflows: pin Actions to commit SHAs (tags kept as comments)
- untrack photos/.DS_Store (already gitignored)
</commit_message>
<xml_diff>
--- a/updates/members/aaliyah-chang/info.xlsx
+++ b/updates/members/aaliyah-chang/info.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Member" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Member" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -527,7 +527,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>aaliyah.chang@queensu.ca</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr"/>

</xml_diff>

<commit_message>
members: add Sophia Thurston, Hassaan photo/role; contact UX final; maintenance
Visible:
- members: Sophia Thurston (MASc Fall 2026 - Pres) with photo; Hassaan
  Tayyab -> Research Assistant (Jun 2026 - Pres) + real photo; Yawar
  hobbies; single 10-member grid, bold role titles (update_site.py)
- contact: navbar Contact us button top-right on all pages; home contact
  panel with single button (subject 'Lab inquiry'); student inquiries
  point to Teaching page button (subject 'Student inquiry')

Maintenance (invisible):
- updates/members spreadsheets: real member emails -> TBD (they were
  publicly downloadable via the Pages deploy)
- SRI integrity on Bootstrap JS (5 pages), rel=noopener on external
  links, safeUrl() for publication links, Actions pinned to SHAs,
  photos/.DS_Store untracked, html.escape in member rendering
</commit_message>
<xml_diff>
--- a/updates/members/aaliyah-chang/info.xlsx
+++ b/updates/members/aaliyah-chang/info.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Member" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Member" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -527,7 +527,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>aaliyah.chang@queensu.ca</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr"/>

</xml_diff>